<commit_message>
Sweep TitleMapping: fix EA false-positive + 2 under-levelled synonyms
Follow-up audit of all 187 TitleMapping synonyms through the live matcher:

- Guard fix: 'Executive Assistant to CEO/CFO/CTO/CHRO' were wrongly
  flagged as C-suite by the new guard (bare token match) and forced to
  needs-review, though they correctly map to Operations Coordinator.
  _is_c_suite_title now excludes assistant/secretary/'to the X' support
  titles.
- Data: remap 'Head of Digital' -> Head of Marketing and 'Head of
  Finance and Operations' -> Head of Finance (were pointing at Senior
  Manager roles despite the 'Head of' Lead signal).

Result: 0 of 187 synonyms would be flagged by the live matcher; validates
0 errors / 0 warnings.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ZYr5d8XhRVzzHT3E1vLip
</commit_message>
<xml_diff>
--- a/jobsy_reference_library.xlsx
+++ b/jobsy_reference_library.xlsx
@@ -52122,7 +52122,7 @@
       </c>
       <c r="B174" s="10" t="inlineStr">
         <is>
-          <t>J-FIN-05</t>
+          <t>J-FIN-06</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -52418,7 +52418,7 @@
       </c>
       <c r="B182" s="10" t="inlineStr">
         <is>
-          <t>J-MKT-03</t>
+          <t>J-MKT-05</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">

</xml_diff>

<commit_message>
Fix two matches found by tricky-title drive: NL + typo resilience
Driving the app with tricky titles surfaced two bad fuzzy matches:
- 'Financieel Directeur' (NL: Finance Director) -> Head of HR
- 'Senior Developper' (typo) -> Senior Customer Success Manager

Fixes:
- TitleMapping: add Dutch/robust synonyms (Financieel Directeur -> Head of
  Finance, Financieel Manager, Hoofd Financiën, Senior Developer,
  Ontwikkelaar, Software Ontwikkelaar).
- Matcher function guard: add NL/typo keywords (financieel, boekhoud,
  ontwikkelaar, developper) so fuzzy hits in the wrong domain are rejected.

Now: Financieel Directeur -> Head of Finance; Senior Developper -> Senior
Software Engineer. Validates 0 errors / 0 warnings.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ZYr5d8XhRVzzHT3E1vLip
</commit_message>
<xml_diff>
--- a/jobsy_reference_library.xlsx
+++ b/jobsy_reference_library.xlsx
@@ -45706,7 +45706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G188"/>
+  <dimension ref="A1:G193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -52664,6 +52664,191 @@
         </is>
       </c>
       <c r="G188" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Financieel Directeur</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>J-FIN-06</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Seed v1 (nl)</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Financieel Manager</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>J-FIN-05</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Seed v1 (nl)</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Senior Developer</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>J-ENG-03</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Seed v1 (nl)</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Software Ontwikkelaar</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>J-ENG-02</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Seed v1 (nl)</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Directeur Operations</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>J-OPS-05</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Seed v1 (nl)</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>

</xml_diff>

<commit_message>
Recalibrate baseline salary bands to NL 2026 market data
The industry factors and pay mix were grounded in published data, but the
baseline SalaryBands were seed estimates. Validate the highest-impact
bands against 2026 figures (Robert Walters / Robert Half guides + tech pay
aggregators) and lift the ones that were materially low:

- Engineering Senior P50 EUR87k -> EUR95k (senior SWE base EUR90-104k)
- Data Senior P50 EUR79k -> EUR86k (data scientist avg ~EUR101k)
- Finance Medior P50 EUR50k -> EUR53k (accountant avg EUR67k, entry EUR48k)
- Product Junior P50 EUR49k -> EUR55k (PM entry EUR57.5k)
- Engineering Medior P50 EUR64k -> EUR66k (mid tech ~EUR74k TC)

Already-aligned bands were left unchanged to avoid unsourced churn; the
validation source is recorded in SalarySources. Validates 0/0; all 49
tests pass (band min<=p50<=max guard holds).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ZYr5d8XhRVzzHT3E1vLip
</commit_message>
<xml_diff>
--- a/jobsy_reference_library.xlsx
+++ b/jobsy_reference_library.xlsx
@@ -53108,7 +53108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -53352,6 +53352,38 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>Industry-level pay factors are calibrated to CBS sector wage relativities and public NL salary guides (2026). Function-within-industry tilts are informed estimates. Factors multiply the baseline SalaryBands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Role base-salary validation 2026 (Eng, Data, Finance, Product)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Robert Walters / Robert Half + tech pay aggregators</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Salary guide + aggregators</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.robertwalters.nl/en/our-services/salary-survey.html</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Baseline SalaryBands for senior tech, data, accountant and APM roles</t>
         </is>
       </c>
     </row>
@@ -56787,19 +56819,19 @@
         <v>6</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>42000</v>
+        <v>45000</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>46000</v>
+        <v>49000</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>50000</v>
+        <v>53000</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>54000</v>
+        <v>57000</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>58000</v>
+        <v>62000</v>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
@@ -56808,7 +56840,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Seed v1</t>
+          <t>Validated to NL 2026 market (Robert Walters / Robert Half guides + tech pay aggregators)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -56828,7 +56860,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -57027,19 +57059,19 @@
         <v>6</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>54000</v>
+        <v>55000</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>59000</v>
+        <v>61000</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>64000</v>
+        <v>66000</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>69000</v>
+        <v>71000</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>74000</v>
+        <v>78000</v>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
@@ -57048,7 +57080,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Seed v1</t>
+          <t>Validated to NL 2026 market (Robert Walters / Robert Half guides + tech pay aggregators)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -57068,7 +57100,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -57087,19 +57119,19 @@
         <v>10</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>74000</v>
+        <v>80000</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>80000</v>
+        <v>87000</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>87000</v>
+        <v>95000</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>94000</v>
+        <v>105000</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>100000</v>
+        <v>115000</v>
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
@@ -57108,7 +57140,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Seed v1</t>
+          <t>Validated to NL 2026 market (Robert Walters / Robert Half guides + tech pay aggregators)</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -57128,7 +57160,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -57267,19 +57299,19 @@
         <v>9</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>66000</v>
+        <v>70000</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>72000</v>
+        <v>78000</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>79000</v>
+        <v>86000</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>86000</v>
+        <v>94000</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>92000</v>
+        <v>102000</v>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
@@ -57288,7 +57320,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Seed v1</t>
+          <t>Validated to NL 2026 market (Robert Walters / Robert Half guides + tech pay aggregators)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -57308,7 +57340,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -57387,19 +57419,19 @@
         <v>3</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>42000</v>
+        <v>48000</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>46000</v>
+        <v>51000</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>49000</v>
+        <v>55000</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>52000</v>
+        <v>58000</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>56000</v>
+        <v>62000</v>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
@@ -57408,7 +57440,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Seed v1</t>
+          <t>Validated to NL 2026 market (Robert Walters / Robert Half guides + tech pay aggregators)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -57428,7 +57460,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>

</xml_diff>